<commit_message>
Branch A: build Microsoft Lists workflow + apply confirmed decisions
- Assigned Driver = Choice of 4 roles (Driver 1/2, FACT Coordinator, Supervisor)
- FACT/Lyft = simple Yes/No flag; excluded from driver emails, own view
- Notifications = per-driver Outlook email primary (Teams optional)
- Regenerate + revalidate import workbook; update schema, views, flow, templates
- Update change-summary HTML page
</commit_message>
<xml_diff>
--- a/branch-a-lists/Schedule for Lists Import.xlsx
+++ b/branch-a-lists/Schedule for Lists Import.xlsx
@@ -174,7 +174,7 @@
     <tableColumn id="7" name="Destination"/>
     <tableColumn id="8" name="Return Time"/>
     <tableColumn id="9" name="Assigned Driver"/>
-    <tableColumn id="10" name="Ride Provider"/>
+    <tableColumn id="10" name="Outside Ride (FACT/Lyft)"/>
     <tableColumn id="11" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -482,7 +482,7 @@
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -534,7 +534,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Ride Provider</t>
+          <t>Outside Ride (FACT/Lyft)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -580,14 +580,14 @@
       <c r="H2" s="4" t="n">
         <v>46188.53125</v>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Robert Nguyen</t>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Driver 1</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -633,14 +633,14 @@
       <c r="H3" s="4" t="n">
         <v>46188.54166666666</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Robert Nguyen</t>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Driver 1</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr"/>
@@ -682,14 +682,14 @@
       <c r="H4" s="4" t="n">
         <v>46188.53125</v>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Maria Lopez</t>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Driver 2</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -735,14 +735,14 @@
       <c r="H5" s="4" t="n">
         <v>46188.54166666666</v>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Maria Lopez</t>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Driver 2</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -788,14 +788,14 @@
       <c r="H6" s="4" t="n">
         <v>46188.53125</v>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Robert Nguyen</t>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Driver 1</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -837,14 +837,14 @@
       <c r="H7" s="4" t="n">
         <v>46188.54166666666</v>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Maria Lopez</t>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Driver 2</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -890,14 +890,14 @@
       <c r="H8" s="4" t="n">
         <v>46188.53125</v>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Robert Nguyen</t>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Driver 1</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
@@ -939,14 +939,14 @@
       <c r="H9" s="4" t="n">
         <v>46188.54166666666</v>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Maria Lopez</t>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>FACT Coordinator</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>FACT</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -992,14 +992,14 @@
       <c r="H10" s="4" t="n">
         <v>46188.53125</v>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Robert Nguyen</t>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Driver 1</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1043,14 +1043,14 @@
         </is>
       </c>
       <c r="H11" s="3" t="n"/>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>Maria Lopez</t>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>FACT Coordinator</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Lyft</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">

</xml_diff>